<commit_message>
Corrección de formato pdf
</commit_message>
<xml_diff>
--- a/backend/preview_out.xlsx
+++ b/backend/preview_out.xlsx
@@ -68,7 +68,7 @@
     <t>TIEMPO DE ENTREGA:</t>
   </si>
   <si>
-    <t>FECHA:</t>
+    <t>FECHA DE LA OFERTA:</t>
   </si>
   <si>
     <t>11 de agosto de 2026</t>
@@ -602,7 +602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -658,13 +658,13 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -677,7 +677,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -696,7 +696,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -706,7 +706,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -745,22 +745,22 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="5" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -786,6 +786,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1643,79 +1649,79 @@
       <c r="G30" s="53"/>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="58" t="s">
+      <c r="A31" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="58"/>
-      <c r="C31" s="58"/>
-      <c r="D31" s="58"/>
-      <c r="E31" s="58"/>
-      <c r="F31" s="58"/>
-      <c r="G31" s="58"/>
+      <c r="B31" s="60"/>
+      <c r="C31" s="60"/>
+      <c r="D31" s="60"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="60"/>
+      <c r="G31" s="60"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="58" t="s">
+      <c r="A32" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="B32" s="58"/>
-      <c r="C32" s="58"/>
-      <c r="D32" s="58"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="58"/>
-      <c r="G32" s="58"/>
+      <c r="B32" s="61"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="61"/>
+      <c r="G32" s="61"/>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="58" t="s">
+      <c r="A33" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="58"/>
-      <c r="G33" s="58"/>
+      <c r="B33" s="61"/>
+      <c r="C33" s="61"/>
+      <c r="D33" s="61"/>
+      <c r="E33" s="61"/>
+      <c r="F33" s="61"/>
+      <c r="G33" s="61"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="58" t="s">
+      <c r="A34" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="58"/>
-      <c r="C34" s="58"/>
-      <c r="D34" s="58"/>
-      <c r="E34" s="58"/>
-      <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="58" t="s">
+      <c r="A35" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="58"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="58"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="58" t="s">
+      <c r="A36" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="B36" s="58"/>
-      <c r="C36" s="58"/>
-      <c r="D36" s="58"/>
-      <c r="E36" s="58"/>
-      <c r="F36" s="58"/>
-      <c r="G36" s="58"/>
+      <c r="B36" s="61"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="60"/>
-      <c r="B37" s="61"/>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="62"/>
+      <c r="A37" s="62"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="63"/>
+      <c r="F37" s="63"/>
+      <c r="G37" s="64"/>
     </row>
     <row r="38" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>